<commit_message>
feat: fold NORTHEDGE ai-forum lessons into AI-DLC offering
- Delivery & Operations: rubric now reflects AI-first lifecycle shift (design-up-front, clarity of intent as multiplier, bottleneck shift)
- Culture & Adoption: Four Fears framework integrated as diagnostic tool, middle-layer bottleneck questions added
- Workshop HTML: economics callout on results page, 8-week prove-it model for embedded team, expanded workshop modules
- Service Catalogue: enhanced qualifying questions (release cadence, coordination roles, prior AI tooling attempts), expanded discovery questions per dimension, 8-week FDE structure, Key Frameworks section (Four Fears, AI-First Lifecycle, Middle Layer Bottleneck, Economics, Prove-It Model), detailed per-module attendee guidance
</commit_message>
<xml_diff>
--- a/analysis/D55/ai-dlc/spreadsheets/AI-DLC Service Catalogue.xlsx
+++ b/analysis/D55/ai-dlc/spreadsheets/AI-DLC Service Catalogue.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C37"/>
+  <dimension ref="B1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,8 @@
         <is>
           <t>• Have you started using AI in any capacity (even experimentation)?
 • Is there executive sponsorship or budget for AI initiatives?
-• Do you have data/ML practitioners on staff, or is it outsourced?</t>
+• Do you have data/ML practitioners on staff, or is it outsourced?
+• Have you tried AI developer tooling (Copilot, Claude, etc.)? What happened?</t>
         </is>
       </c>
     </row>
@@ -562,7 +563,8 @@
         <is>
           <t>• Where does AI sit on the board agenda? Is there a deadline or trigger?
 • Are competitors doing things with AI that worry you?
-• Is there a compliance trigger (EU AI Act, sector regulation)?</t>
+• Is there a compliance trigger (EU AI Act, sector regulation)?
+• What's changed in the last 6–12 months that makes this conversation worth having now?</t>
         </is>
       </c>
     </row>
@@ -575,8 +577,10 @@
       <c r="C15" s="5" t="inlineStr">
         <is>
           <t>• How many people would be involved in or affected by AI adoption?
+• Do you have heavy coordination roles (POs, BAs, PMs)? How many vs engineers?
 • How many data sources and systems are in play?
-• What's your current cloud platform, and is that settled?</t>
+• What's your current cloud platform, and is that settled?
+• What's your release cadence today? Days, weeks, months?</t>
         </is>
       </c>
     </row>
@@ -590,7 +594,8 @@
         <is>
           <t>• Is there budget allocated for AI strategy or implementation work?
 • Who makes the decision to engage external support?
-• What does 'decided' look like for you, and by when?</t>
+• What does 'decided' look like for you, and by when?
+• Would you prefer to buy a strategy/roadmap, or buy people and time?</t>
         </is>
       </c>
     </row>
@@ -617,7 +622,7 @@
           <t>• Who owns AI in your organisation? Is there an executive sponsor?
 • Can you point to a document linking AI initiatives to business outcomes?
 • How are AI projects prioritised? What gets funded and why?
-• If AI budgets were cut tomorrow, who'd fight for them?</t>
+• If AI budgets were cut tomorrow, who'd fight for them and with what evidence?</t>
         </is>
       </c>
     </row>
@@ -632,7 +637,8 @@
           <t>• Where does your data live today? How many systems for a full picture?
 • Do you have a data catalogue? Do people actually use it?
 • How long to produce a clean joined dataset across key entities?
-• What's your biggest data quality pain point?</t>
+• What's your biggest data quality pain point?
+• AI on bad data produces bad outputs faster — how confident are you in your data foundation?</t>
         </is>
       </c>
     </row>
@@ -647,7 +653,8 @@
           <t>• How many tools does a practitioner touch in a typical week?
 • What's the journey from idea to production? How many hand-offs?
 • If a new joiner started tomorrow, how long before productive?
-• What's your biggest frustration with current tooling?</t>
+• What's your biggest frustration with current tooling?
+• Are your devs using AI-assisted tooling (Copilot, Claude, agentic IDEs)? What's the experience?</t>
         </is>
       </c>
     </row>
@@ -661,6 +668,7 @@
         <is>
           <t>• How many people on data/AI full-time vs second hat?
 • When a senior leaves, what breaks? How long to backfill?
+• Who's the bottleneck today? What are they spending their time on?
 • Is there a training programme for AI? Who's been through it?
 • If you could add three roles tomorrow, what and why?</t>
         </is>
@@ -677,7 +685,8 @@
           <t>• Do you have an AI usage policy? Who enforces it?
 • How do you document what a model does and what decisions it influences?
 • Are you aware of EU AI Act implications for your use cases?
-• If a regulator asked 'show me how this decision was made' — could you?</t>
+• If a regulator asked 'show me how this decision was made' — could you?
+• Are workloads running in the correct region? Is access locked down?</t>
         </is>
       </c>
     </row>
@@ -692,7 +701,9 @@
           <t>• How many models in production? How did they get there?
 • What happens when model performance degrades?
 • What's the gap between experiments and what's shipping?
-• 'Deploy this by Friday' — realistic or laughable?</t>
+• 'Deploy this by Friday' — realistic or laughable?
+• How much time in design/spec vs implementation? Has that changed with AI tooling?
+• When devs go faster, where does the bottleneck shift — specs? Reviews? Coordination?</t>
         </is>
       </c>
     </row>
@@ -706,7 +717,8 @@
         <is>
           <t>• Do you know AI/data spend per team or project?
 • Last time finance asked 'what are we getting?' — what was the answer?
-• How do you decide to continue, scale, or kill an AI initiative?</t>
+• How do you decide to continue, scale, or kill an AI initiative?
+• AI tooling costs ~£150–200/seat/month for ~5x productivity — have you done this maths for your team?</t>
         </is>
       </c>
     </row>
@@ -718,9 +730,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>• How do non-technical staff feel about AI?
+          <t>• How do non-technical staff feel about AI? Excited? Threatened? Indifferent?
 • Are there AI tools in use outside the data/tech team?
-• If a frontline employee had an AI idea, who would they tell?</t>
+• If a frontline employee had an AI idea, who would they tell?
+• Where is resistance coming from? Which roles or personality types push back?
+• When devs adopted AI and went faster, did coordination roles (POs/BAs/PMs) keep pace or become a bottleneck?
+• Has anyone left or been moved because they couldn't adapt?</t>
         </is>
       </c>
     </row>
@@ -759,11 +774,17 @@
           <t>1. Discovery &amp; Strategy Session (DSD) — £30–50k
    Fully costed AI/data strategy + roadmap. Pure consultancy. 4–6 weeks.
 2. Prescriptive Workshops — £5–15k per module
-   How to spec | Developer tooling | Compliance &amp; governance | MLOps | Process &amp; ceremonies | Data platform | Cost optimisation
+   Modules: AI Strategy | AI-First Delivery Lifecycle (how to spec, contracts upfront, ceremony changes) | Developer Tooling | Compliance &amp; Governance | MLOps | Process &amp; Ceremonies | Data Platform | Cost Optimisation | Four Fears (Culture &amp; Change)
 3. Embedded Team / FDEs — £15–25k per engineer/month
-   Forward deployed engineers alongside customer team. Build + upskill.
+   8-week prove-it model:
+   • Weeks 1–2: Assess codebase, tooling, current AI adoption, identify quick wins
+   • Weeks 3–6: Embed in a squad, apply AI-first delivery on real work, track metrics from day one
+   • Weeks 7–8: Demonstrate improvement with numbers, produce playbooks, deliver rollout plan
+   D55 embeds, proves, then enables. Not a permanent dependency.
+   Once one squad is working, use it as reference to pull others forward.
 4. Runbook &amp; Asset Delivery — from £20k (or included with DSD)
-   Prescriptive step-by-step guide with decision points and options.</t>
+   Prescriptive step-by-step guide with decision points and options.
+   The runbook IS the asset — tells them exactly how to get from A to B.</t>
         </is>
       </c>
     </row>
@@ -780,12 +801,15 @@
         <is>
           <t>• Clarity in 1 hour — know exactly where you stand and what to do next
 • No upfront cost — assessment is free, you choose what (if anything) to buy
-• Visual gap analysis makes the case for investment to leadership
+• Visual gap analysis makes the case for investment to leadership/PE/board
 • Roadmap is actionable — phased, prioritised, with clear deliverables
 • Flexible engagement — buy consultancy, workshops, or embedded people
-• Knowledge transfer built in — we upskill as we deliver
+• Knowledge transfer built in — we upskill as we deliver, not a permanent dependency
 • Prescriptive not theoretical — runbooks with specific steps, not just advice
-• AWS-native solutions with cost advantage over Snowflake/Databricks</t>
+• AWS-native solutions with cost advantage over Snowflake/Databricks
+• Proven economics: ~£150–200/seat/month AI tooling delivers ~5x developer productivity
+  For a 50-person team: ~£120k/year in tooling for output equivalent to 200+ engineers
+  The real cost is delay, not investment</t>
         </is>
       </c>
     </row>
@@ -805,10 +829,11 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>• CTO / VP Engineering / Head of Data (decision maker)
+          <t>• CTO / VP Engineering / Head of Data (decision maker + strategy perspective)
 • Senior data/ML engineer (technical reality check)
 • Someone from finance or ops (cost/value perspective)
-Optional: Product owner or business stakeholder</t>
+• Product owner or business stakeholder (adoption/culture lens)
+3–5 people. Enough perspectives to score honestly, few enough to have a real conversation.</t>
         </is>
       </c>
     </row>
@@ -820,9 +845,126 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>• Varies by module — dev tooling needs engineers, governance needs legal/compliance
-• Typically 4–10 people per workshop
-• Mix of doers and decision makers</t>
+          <t>Varies by module:
+• AI-First Delivery Lifecycle: Engineering leads, POs, Scrum Masters, BAs (the people whose process changes)
+• Developer Tooling: Senior engineers, tech leads (hands-on practitioners)
+• Compliance &amp; Governance: CTO, legal/compliance, security, data protection
+• Four Fears / Culture: Leadership team, HR, people who'll champion or block adoption
+• MLOps: Data engineers, ML engineers, platform/infra team
+• Cost Optimisation: Finance, engineering leads, FinOps (if exists)
+Typically 4–10 people per workshop. Mix of doers and decision makers.
+Key learning from experience: include the 'middle layer' (POs/BAs/PMs) early — they become the bottleneck when devs go faster and need to adapt too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>KEY FRAMEWORKS &amp; INSIGHTS</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>(Proven in delivery — used during assessment and workshops)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Four Fears Framework</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Diagnostic tool for AI adoption resistance. Four personality types, four fears:
+• Controller (tasks/past): 'I can't manage what I can't understand' → Reframe: AI gives MORE oversight and observability, not less
+• Driver (tasks/future): 'This could go wrong and I'll be accountable' → Reframe: AI compresses feedback loops, you fail faster and cheaper
+• Stabiliser (people/past): 'My position and authority are under threat' → Reframe: People who orchestrate AI become MORE valuable
+• Influencer (people/future): 'If AI does the impressive stuff, what's my value?' → Reframe: AI handles grunt work, you get more stage
+Application: diagnose which fears dominate, tailor intervention per role/person. Common pattern: POs/BAs/PMs are typically Controllers + Stabilisers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>AI-First Delivery Lifecycle</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Key insight: when implementation is 5x faster, the bottleneck shifts to clarity of intent.
+The lifecycle shifts toward design-up-front (NOT waterfall):
+1. Analysis &amp; Design — more time here than traditional agile. Clear specs.
+2. Contracts &amp; Integration Points — understand touch points upfront.
+3. Implementation — devs with agentic tooling against well-defined specs.
+4. Testing — human-in-the-loop + automated (Playwright MCP for regression).
+5. Documentation &amp; Handover — AI-generated assets.
+Garbage specs at 5x speed = garbage 5x faster. Design discipline is the multiplier on the multiplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Middle Layer Bottleneck</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>When devs go 5x faster with AI tooling, coordination roles can't keep pace:
+• POs can't write specs fast enough
+• BAs can't break down requirements fast enough
+• PMs can't coordinate fast enough
+They become the constraint. Unblocked by:
+• Action first, metrics to prove it, regular retros
+• 1-on-1 training and support for those roles
+• AI-assisted spec writing and prioritisation
+• Not everyone will come around — plan for it, budget time for it</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>The Economics</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>• AI developer tooling: ~£150–200/seat/month (Copilot + Claude + IDE)
+• Observed productivity gain: ~5x (with belief this improves further)
+• For 50 engineers: ~£120k/year in tooling for output of 200+ engineers
+• Even at 20% headcount efficiency, that's millions in savings
+• No expensive infrastructure or custom model training required
+• The real cost is DELAY, not investment
+PE/CFO framing: AI-native engineering org is a valuation multiplier at exit. Output per £ of engineering cost is the metric that matters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>8-Week Prove-It Model</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Structured embedded engagement (default shape for FDE work):
+Weeks 1–2: ASSESS
+• Assess codebase, tooling, current AI adoption
+• Understand resistance patterns (Four Fears)
+• Identify quick wins and high-friction areas
+Weeks 3–6: PROVE
+• Embed D55 people in an existing squad (or stand up fresh D55-led squad)
+• Apply AI-first delivery on a real piece of work
+• Track metrics from day one (PRs, cycle time, deployment frequency)
+Weeks 7–8: TRANSLATE
+• Demonstrate improvement with hard numbers
+• Translate ways of working into reusable assets (guides, patterns, configs)
+• Produce rollout plan for other squads
+Then: one squad is the reference point to pull others forward. Assets and playbooks allow teams to self-serve after D55 steps back.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: regenerate spreadsheets for AI-for-development focus
- Value Proposition Canvas: pain points now specific to AI-assisted engineering (patchy adoption, garbage specs, middle-layer bottleneck, governance gaps, resistance, can't prove ROI)
- Service Catalogue: dimensions, qualifying questions, services all aligned to development lifecycle focus
- Critique output updated (PASS: CTO 4/5, Marketing 3/5)
</commit_message>
<xml_diff>
--- a/analysis/D55/ai-dlc/spreadsheets/AI-DLC Service Catalogue.xlsx
+++ b/analysis/D55/ai-dlc/spreadsheets/AI-DLC Service Catalogue.xlsx
@@ -467,7 +467,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>D55 AI Development Lifecycle Assessment &amp; Delivery Services</t>
+          <t>AI in the Development Lifecycle — Assessment &amp; Delivery Services</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>A free, structured 1-hour assessment workshop that scores an organisation across 8 AI maturity dimensions (Strategy, Data, Tooling, Team, Governance, Delivery, Cost, Culture). Produces a radar chart showing current state vs target state, a gap analysis with recommended services, and an indicative runbook. The output drives further paid engagements.</t>
+          <t>A free, structured 1-hour assessment that scores an engineering organisation across 8 dimensions of AI-assisted development readiness: Leadership &amp; Mandate, Developer Tooling, Specification &amp; Design, Delivery Process, Testing &amp; Quality, Governance &amp; Security, Team Adaptation, and Metrics &amp; ROI. Produces a radar chart, gap analysis, and indicative roadmap. The output drives further paid engagements.</t>
         </is>
       </c>
     </row>
@@ -503,12 +503,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>• Mid-market / SME (250–2000 employees)
-• Some AI experimentation but struggling to scale or show ROI
-• Leadership bought into AI but unclear on strategy or next steps
-• May have data platform but AI workloads not in production
-• Feeling pressure from competitors, regulation, or board
-• On AWS or open to AWS (for service delivery alignment)</t>
+          <t>• Mid-market engineering org (20–200 developers)
+• On AWS (or committed to AWS)
+• Have purchased or are considering AI dev tooling (Copilot, Claude, etc.)
+• Struggling with: patchy adoption, can't prove ROI, process hasn't adapted, or resistance from parts of the team
+• Executive sponsor exists (CTO/VP Eng) who wants this to work
+• PE-backed or board-level pressure for engineering efficiency preferred</t>
         </is>
       </c>
     </row>
@@ -520,13 +520,12 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>• No clear AI strategy tied to business outcomes
-• Tool and platform sprawl — high friction, long onboarding
-• AI work stuck in experimentation, not reaching production
-• No governance framework — EU AI Act exposure unknown
-• Can't quantify AI spend or demonstrate ROI to finance
-• Skills concentrated in individuals, no scalable capability
-• Culture not ready — AI seen as tech team's problem, not business-wide</t>
+          <t>• Bought licences but adoption is patchy — ROI unclear
+• Devs faster but quality inconsistent — specs haven't adapted
+• POs/BAs/PMs becoming bottlenecks — process unchanged
+• No governance — data leaking into AI tools, no audit trail
+• Resistance from seniors or coordination roles — adoption stalling
+• Can't quantify the gain — 'it feels faster' but no numbers for the board</t>
         </is>
       </c>
     </row>
@@ -541,201 +540,173 @@
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AI Maturity</t>
+          <t>Tooling Status</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>• Have you started using AI in any capacity (even experimentation)?
-• Is there executive sponsorship or budget for AI initiatives?
-• Do you have data/ML practitioners on staff, or is it outsourced?
-• Have you tried AI developer tooling (Copilot, Claude, etc.)? What happened?</t>
+          <t>• Are developers currently using AI-assisted coding tools? Which ones?
+• How long have they been in use? Enterprise or individual licences?
+• What percentage of developers are actively using them?</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Ambition &amp; Urgency</t>
+          <t>Adoption &amp; Pain</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>• Where does AI sit on the board agenda? Is there a deadline or trigger?
-• Are competitors doing things with AI that worry you?
-• Is there a compliance trigger (EU AI Act, sector regulation)?
-• What's changed in the last 6–12 months that makes this conversation worth having now?</t>
+          <t>• What's working well? What's not?
+• Have you seen productivity improvements? Can you quantify them?
+• Is there resistance? From whom?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Scale &amp; Complexity</t>
+          <t>Mandate &amp; Budget</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>• How many people would be involved in or affected by AI adoption?
-• Do you have heavy coordination roles (POs, BAs, PMs)? How many vs engineers?
-• How many data sources and systems are in play?
-• What's your current cloud platform, and is that settled?
-• What's your release cadence today? Days, weeks, months?</t>
+          <t>• Is there executive sponsorship for AI-assisted development specifically?
+• Is there budget for consulting/implementation support?
+• What does 'success' look like for you in 12 months?</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Budget &amp; Decision</t>
+          <t>Disqualifiers</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>• Is there budget allocated for AI strategy or implementation work?
-• Who makes the decision to engage external support?
-• What does 'decided' look like for you, and by when?
-• Would you prefer to buy a strategy/roadmap, or buy people and time?</t>
+          <t>• Fewer than 20 engineers → too small for embedded model
+• Not on AWS and no plans to move → our delivery is AWS-native
+• No executive sponsor AND no budget → can't act on the output
+• Already engaged with another consultancy on same scope → redirect</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>DISCOVERY QUESTIONS</t>
+          <t>WORKSHOP DIMENSIONS</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>(Used during the workshop itself)</t>
+          <t>(8 dimensions assessed during the 1-hour session)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Strategy &amp; Alignment</t>
+          <t>1. Leadership &amp; Mandate</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>• Who owns AI in your organisation? Is there an executive sponsor?
-• Can you point to a document linking AI initiatives to business outcomes?
-• How are AI projects prioritised? What gets funded and why?
-• If AI budgets were cut tomorrow, who'd fight for them and with what evidence?</t>
+          <t>• Who sponsors AI-assisted development? Optional, encouraged, or mandated?
+• Has the investment case been made to finance/board?</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Data Readiness</t>
+          <t>2. Developer Tooling &amp; Adoption</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>• Where does your data live today? How many systems for a full picture?
-• Do you have a data catalogue? Do people actually use it?
-• How long to produce a clean joined dataset across key entities?
-• What's your biggest data quality pain point?
-• AI on bad data produces bad outputs faster — how confident are you in your data foundation?</t>
+          <t>• What tools are in use? What % use daily? Standard config or ad-hoc?
+• Gap between best adopter and least engaged?</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Tooling &amp; Platform</t>
+          <t>3. Specification &amp; Design</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>• How many tools does a practitioner touch in a typical week?
-• What's the journey from idea to production? How many hand-offs?
-• If a new joiner started tomorrow, how long before productive?
-• What's your biggest frustration with current tooling?
-• Are your devs using AI-assisted tooling (Copilot, Claude, agentic IDEs)? What's the experience?</t>
+          <t>• Time in design vs implementation — has the ratio changed?
+• Are specs written for AI consumption? Contracts defined upfront?</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Team &amp; Capability</t>
+          <t>4. Delivery Process &amp; Ceremonies</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>• How many people on data/AI full-time vs second hat?
-• When a senior leaves, what breaks? How long to backfill?
-• Who's the bottleneck today? What are they spending their time on?
-• Is there a training programme for AI? Who's been through it?
-• If you could add three roles tomorrow, what and why?</t>
+          <t>• Have ceremonies adapted? Where are the new bottlenecks?
+• Can POs/BAs keep pace with developer velocity?</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Governance &amp; Compliance</t>
+          <t>5. Testing &amp; Quality</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>• Do you have an AI usage policy? Who enforces it?
-• How do you document what a model does and what decisions it influences?
-• Are you aware of EU AI Act implications for your use cases?
-• If a regulator asked 'show me how this decision was made' — could you?
-• Are workloads running in the correct region? Is access locked down?</t>
+          <t>• How is AI-generated code validated? Same bar as human code?
+• Automated regression? Human-in-the-loop at integration points?</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Delivery &amp; Operations</t>
+          <t>6. Governance, Security &amp; Compliance</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>• How many models in production? How did they get there?
-• What happens when model performance degrades?
-• What's the gap between experiments and what's shipping?
-• 'Deploy this by Friday' — realistic or laughable?
-• How much time in design/spec vs implementation? Has that changed with AI tooling?
-• When devs go faster, where does the bottleneck shift — specs? Reviews? Coordination?</t>
+          <t>• AI usage policy? DLP controls? Enterprise agreements?
+• Code provenance tracking? EU AI Act classification?</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Cost &amp; Value</t>
+          <t>7. Team Adaptation &amp; Skills</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>• Do you know AI/data spend per team or project?
-• Last time finance asked 'what are we getting?' — what was the answer?
-• How do you decide to continue, scale, or kill an AI initiative?
-• AI tooling costs ~£150–200/seat/month for ~5x productivity — have you done this maths for your team?</t>
+          <t>• Where is resistance? Which roles? (Use Four Fears to diagnose)
+• Training programme? Middle layer adapting or bottlenecking?</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Culture &amp; Adoption</t>
+          <t>8. Metrics &amp; ROI</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>• How do non-technical staff feel about AI? Excited? Threatened? Indifferent?
-• Are there AI tools in use outside the data/tech team?
-• If a frontline employee had an AI idea, who would they tell?
-• Where is resistance coming from? Which roles or personality types push back?
-• When devs adopted AI and went faster, did coordination roles (POs/BAs/PMs) keep pace or become a bottleneck?
-• Has anyone left or been moved because they couldn't adapt?</t>
+          <t>• What evidence exists? Cycle time, PRs, deploys, defects?
+• Can you make the case to the CFO/board in £ terms?</t>
         </is>
       </c>
     </row>
@@ -759,7 +730,8 @@
 • Gap analysis with severity scoring
 • Recommended services mapped to each gap
 • Indicative runbook (phased by priority)
-• Engagement model recommendation</t>
+• Engagement model recommendation
+• Written summary with direct quotes and narrative (within 48 hours)</t>
         </is>
       </c>
     </row>
@@ -771,20 +743,17 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>1. Discovery &amp; Strategy Session (DSD) — £30–50k
-   Fully costed AI/data strategy + roadmap. Pure consultancy. 4–6 weeks.
+          <t>1. Discovery &amp; Strategy Session — £30–50k
+   Costed roadmap for org-wide AI-assisted development rollout. 4–6 weeks.
 2. Prescriptive Workshops — £5–15k per module
-   Modules: AI Strategy | AI-First Delivery Lifecycle (how to spec, contracts upfront, ceremony changes) | Developer Tooling | Compliance &amp; Governance | MLOps | Process &amp; Ceremonies | Data Platform | Cost Optimisation | Four Fears (Culture &amp; Change)
-3. Embedded Team / FDEs — £15–25k per engineer/month
-   8-week prove-it model:
-   • Weeks 1–2: Assess codebase, tooling, current AI adoption, identify quick wins
-   • Weeks 3–6: Embed in a squad, apply AI-first delivery on real work, track metrics from day one
-   • Weeks 7–8: Demonstrate improvement with numbers, produce playbooks, deliver rollout plan
+   Modules: AI-First Delivery Lifecycle | Developer Tooling Setup | Governance &amp; DLP | Process &amp; Ceremonies | Testing Strategy | Metrics &amp; ROI | Four Fears (Team Change)
+3. Embedded Team / 8-Week Prove-It — £15–25k per engineer/month
+   Weeks 1–2: Assess codebase, tooling, adoption barriers
+   Weeks 3–6: Embed in squad, apply AI-first delivery, track metrics
+   Weeks 7–8: Demonstrate improvement, produce playbooks, rollout plan
    D55 embeds, proves, then enables. Not a permanent dependency.
-   Once one squad is working, use it as reference to pull others forward.
-4. Runbook &amp; Asset Delivery — from £20k (or included with DSD)
-   Prescriptive step-by-step guide with decision points and options.
-   The runbook IS the asset — tells them exactly how to get from A to B.</t>
+4. Runbook &amp; Asset Delivery — from £20k (or included with Discovery)
+   Prescriptive step-by-step playbook: standard configs, skills files, process changes, role definitions, measurement framework. The asset your team follows after we leave.</t>
         </is>
       </c>
     </row>
@@ -799,17 +768,15 @@
     <row r="33">
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>• Clarity in 1 hour — know exactly where you stand and what to do next
-• No upfront cost — assessment is free, you choose what (if anything) to buy
-• Visual gap analysis makes the case for investment to leadership/PE/board
-• Roadmap is actionable — phased, prioritised, with clear deliverables
-• Flexible engagement — buy consultancy, workshops, or embedded people
-• Knowledge transfer built in — we upskill as we deliver, not a permanent dependency
-• Prescriptive not theoretical — runbooks with specific steps, not just advice
-• AWS-native solutions with cost advantage over Snowflake/Databricks
-• Proven economics: ~£150–200/seat/month AI tooling delivers ~5x developer productivity
-  For a 50-person team: ~£120k/year in tooling for output equivalent to 200+ engineers
-  The real cost is delay, not investment</t>
+          <t>• Clarity in 1 hour — know exactly where you stand with AI-assisted development
+• No upfront cost — assessment is free, choose what (if anything) to buy
+• Proven economics: ~£200/seat/month delivers ~3-5x developer productivity
+  For 50 engineers: ~£120k/year for output equivalent to 150-250 engineers
+• 8-week prove-it: see results with real metrics before committing to scale
+• Not a permanent dependency — we produce playbooks and leave
+• Process adapted, not just tools deployed — the second-order effects handled
+• Resistance diagnosed and addressed — not ignored until it blocks adoption
+• The real cost is delay, not investment</t>
         </is>
       </c>
     </row>
@@ -829,11 +796,10 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>• CTO / VP Engineering / Head of Data (decision maker + strategy perspective)
-• Senior data/ML engineer (technical reality check)
-• Someone from finance or ops (cost/value perspective)
-• Product owner or business stakeholder (adoption/culture lens)
-3–5 people. Enough perspectives to score honestly, few enough to have a real conversation.</t>
+          <t>• CTO / VP Engineering (decision maker, mandate perspective)
+• Engineering Manager or Tech Lead (ground-truth on tooling and adoption)
+• A Product Owner or Delivery Lead (process and coordination perspective)
+3–4 people. Enough to score honestly, few enough for real conversation.</t>
         </is>
       </c>
     </row>
@@ -845,126 +811,123 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Varies by module:
-• AI-First Delivery Lifecycle: Engineering leads, POs, Scrum Masters, BAs (the people whose process changes)
-• Developer Tooling: Senior engineers, tech leads (hands-on practitioners)
-• Compliance &amp; Governance: CTO, legal/compliance, security, data protection
-• Four Fears / Culture: Leadership team, HR, people who'll champion or block adoption
-• MLOps: Data engineers, ML engineers, platform/infra team
-• Cost Optimisation: Finance, engineering leads, FinOps (if exists)
-Typically 4–10 people per workshop. Mix of doers and decision makers.
-Key learning from experience: include the 'middle layer' (POs/BAs/PMs) early — they become the bottleneck when devs go faster and need to adapt too.</t>
+          <t>• AI-First Delivery Lifecycle: Engineering leads + POs + Scrum Masters
+• Developer Tooling: Senior engineers, tech leads (hands-on)
+• Governance &amp; DLP: CTO + security + compliance
+• Four Fears / Team Change: Leadership + HR + people who'll champion or block
+• Metrics &amp; ROI: Engineering leads + Finance
+Typically 4–10 people per workshop.
+Key learning: include POs/BAs/PMs early — they become the bottleneck when devs go faster and need to adapt too.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>KEY FRAMEWORKS &amp; INSIGHTS</t>
+          <t>KEY FRAMEWORKS</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>(Proven in delivery — used during assessment and workshops)</t>
+          <t>(Proven in delivery — core IP of this offering)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Four Fears Framework</t>
+          <t>AI-First Delivery Lifecycle</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Diagnostic tool for AI adoption resistance. Four personality types, four fears:
-• Controller (tasks/past): 'I can't manage what I can't understand' → Reframe: AI gives MORE oversight and observability, not less
-• Driver (tasks/future): 'This could go wrong and I'll be accountable' → Reframe: AI compresses feedback loops, you fail faster and cheaper
-• Stabiliser (people/past): 'My position and authority are under threat' → Reframe: People who orchestrate AI become MORE valuable
-• Influencer (people/future): 'If AI does the impressive stuff, what's my value?' → Reframe: AI handles grunt work, you get more stage
-Application: diagnose which fears dominate, tailor intervention per role/person. Common pattern: POs/BAs/PMs are typically Controllers + Stabilisers.</t>
+          <t>When implementation goes 5x faster, clarity of intent becomes the bottleneck.
+The lifecycle shifts toward design-up-front (NOT waterfall):
+1. Analysis &amp; Design — more time here. Clear, structured specs.
+2. Contracts &amp; Integration Points — defined before build.
+3. Implementation — devs with agentic tooling against well-defined specs.
+4. Testing — human-in-the-loop + automated regression.
+5. Documentation — AI-generated assets.
+Garbage specs at 5x speed = garbage 5x faster.
+Design discipline is the multiplier on the multiplier.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>AI-First Delivery Lifecycle</t>
+          <t>Four Fears Framework</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Key insight: when implementation is 5x faster, the bottleneck shifts to clarity of intent.
-The lifecycle shifts toward design-up-front (NOT waterfall):
-1. Analysis &amp; Design — more time here than traditional agile. Clear specs.
-2. Contracts &amp; Integration Points — understand touch points upfront.
-3. Implementation — devs with agentic tooling against well-defined specs.
-4. Testing — human-in-the-loop + automated (Playwright MCP for regression).
-5. Documentation &amp; Handover — AI-generated assets.
-Garbage specs at 5x speed = garbage 5x faster. Design discipline is the multiplier on the multiplier.</t>
+          <t>Diagnostic for AI adoption resistance:
+• Controller: 'I can't manage what I can't understand' → AI gives MORE oversight, not less
+• Driver: 'This could go wrong' → AI compresses feedback loops, fail faster and cheaper
+• Stabiliser: 'My position is threatened' → Orchestrators of AI become MORE valuable
+• Influencer: 'What's my value if AI does the work?' → AI handles grunt work, you get more stage
+Common pattern: POs/BAs/PMs are Controllers + Stabilisers.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Middle Layer Bottleneck</t>
+          <t>Middle-Layer Bottleneck</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>When devs go 5x faster with AI tooling, coordination roles can't keep pace:
+          <t>When devs go 3-5x faster:
 • POs can't write specs fast enough
-• BAs can't break down requirements fast enough
-• PMs can't coordinate fast enough
-They become the constraint. Unblocked by:
-• Action first, metrics to prove it, regular retros
-• 1-on-1 training and support for those roles
-• AI-assisted spec writing and prioritisation
-• Not everyone will come around — plan for it, budget time for it</t>
+• BAs can't break down requirements at pace
+• PMs can't coordinate the new velocity
+They become the constraint. Address by:
+• AI-assisted spec writing for POs
+• Structured templates that reduce ambiguity
+• 1-on-1 coaching and training
+• Process redesign (continuous flow, not batch sprints)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>The Economics</t>
+          <t>8-Week Prove-It Model</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>• AI developer tooling: ~£150–200/seat/month (Copilot + Claude + IDE)
-• Observed productivity gain: ~5x (with belief this improves further)
-• For 50 engineers: ~£120k/year in tooling for output of 200+ engineers
-• Even at 20% headcount efficiency, that's millions in savings
-• No expensive infrastructure or custom model training required
-• The real cost is DELAY, not investment
-PE/CFO framing: AI-native engineering org is a valuation multiplier at exit. Output per £ of engineering cost is the metric that matters.</t>
+          <t>Default shape for embedded engagements:
+Weeks 1–2: ASSESS
+• Assess codebase, tooling, adoption barriers
+• Diagnose resistance patterns (Four Fears)
+• Identify quick wins
+Weeks 3–6: PROVE
+• Embed in a squad, apply AI-first delivery on real work
+• Track metrics from day one
+Weeks 7–8: TRANSLATE
+• Demonstrate improvement with hard numbers
+• Produce reusable playbooks and configs
+• Deliver rollout plan for other squads
+One squad proves it. That squad becomes the reference to pull others forward.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>8-Week Prove-It Model</t>
+          <t>The Economics</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Structured embedded engagement (default shape for FDE work):
-Weeks 1–2: ASSESS
-• Assess codebase, tooling, current AI adoption
-• Understand resistance patterns (Four Fears)
-• Identify quick wins and high-friction areas
-Weeks 3–6: PROVE
-• Embed D55 people in an existing squad (or stand up fresh D55-led squad)
-• Apply AI-first delivery on a real piece of work
-• Track metrics from day one (PRs, cycle time, deployment frequency)
-Weeks 7–8: TRANSLATE
-• Demonstrate improvement with hard numbers
-• Translate ways of working into reusable assets (guides, patterns, configs)
-• Produce rollout plan for other squads
-Then: one squad is the reference point to pull others forward. Assets and playbooks allow teams to self-serve after D55 steps back.</t>
+          <t>• AI dev tooling: ~£150–200/seat/month
+• Observed productivity gain: 3–5x
+• For 50 engineers: ~£120k/year for output of 150–250 engineers
+• The real cost is DELAY, not investment
+PE/CFO framing: AI-native engineering = valuation multiplier at exit.
+Output per £ of engineering cost is the metric that matters.</t>
         </is>
       </c>
     </row>

</xml_diff>